<commit_message>
BARR BBC 2025 subsampling analysis complete
</commit_message>
<xml_diff>
--- a/bbc_subsampleExperiments/2025_BBC_subsampling_BARR.xlsx
+++ b/bbc_subsampleExperiments/2025_BBC_subsampling_BARR.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmeier/Documents/gitRepositories/neon-plant-sampling/bbc_subsampleExperiments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8897D6B7-230E-1B43-AF4B-A4B827D989CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18BD3BAE-8AC3-FD4B-B1FC-09B9A1767377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22520" yWindow="600" windowWidth="27240" windowHeight="28200" xr2:uid="{C2681AD7-DD1C-8E4E-9F7E-0DF192E86DBA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="R_input" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -171,12 +171,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -549,7 +547,7 @@
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2">
         <v>4.4200000000000003E-2</v>
       </c>
     </row>
@@ -566,7 +564,7 @@
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3">
         <v>0</v>
       </c>
     </row>
@@ -583,7 +581,7 @@
       <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4">
         <v>0</v>
       </c>
     </row>
@@ -600,7 +598,7 @@
       <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5">
         <v>0.1711</v>
       </c>
     </row>
@@ -617,7 +615,7 @@
       <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6">
         <v>0</v>
       </c>
     </row>
@@ -634,7 +632,7 @@
       <c r="D7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7">
         <v>0</v>
       </c>
     </row>
@@ -651,7 +649,7 @@
       <c r="D8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8">
         <v>7.6499999999999999E-2</v>
       </c>
     </row>
@@ -668,7 +666,7 @@
       <c r="D9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9">
         <v>0</v>
       </c>
     </row>
@@ -685,7 +683,7 @@
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10">
         <v>0</v>
       </c>
     </row>
@@ -702,7 +700,7 @@
       <c r="D11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11">
         <v>0.47620000000000001</v>
       </c>
     </row>
@@ -719,7 +717,7 @@
       <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12">
         <v>0</v>
       </c>
     </row>
@@ -736,7 +734,7 @@
       <c r="D13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13">
         <v>0</v>
       </c>
     </row>
@@ -753,7 +751,7 @@
       <c r="D14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14">
         <v>0.15679999999999999</v>
       </c>
     </row>
@@ -770,7 +768,7 @@
       <c r="D15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15">
         <v>1.5E-3</v>
       </c>
     </row>
@@ -787,7 +785,7 @@
       <c r="D16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16">
         <v>2.7699999999999999E-2</v>
       </c>
     </row>
@@ -804,7 +802,7 @@
       <c r="D17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17">
         <v>0.1588</v>
       </c>
     </row>
@@ -821,7 +819,7 @@
       <c r="D18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18">
         <v>0</v>
       </c>
     </row>
@@ -838,7 +836,7 @@
       <c r="D19" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E19">
         <v>0</v>
       </c>
     </row>
@@ -855,7 +853,7 @@
       <c r="D20" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20">
         <v>0.24410000000000001</v>
       </c>
     </row>
@@ -872,7 +870,7 @@
       <c r="D21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21">
         <v>0</v>
       </c>
     </row>
@@ -889,7 +887,7 @@
       <c r="D22" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22">
         <v>0</v>
       </c>
     </row>
@@ -906,7 +904,7 @@
       <c r="D23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23">
         <v>1.6026</v>
       </c>
     </row>
@@ -923,7 +921,7 @@
       <c r="D24" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24">
         <v>4.1300000000000003E-2</v>
       </c>
     </row>
@@ -940,7 +938,7 @@
       <c r="D25" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E25">
         <v>0</v>
       </c>
     </row>
@@ -957,7 +955,7 @@
       <c r="D26" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26">
         <v>0.18820000000000001</v>
       </c>
     </row>
@@ -974,7 +972,7 @@
       <c r="D27" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27">
         <v>0</v>
       </c>
     </row>
@@ -991,7 +989,7 @@
       <c r="D28" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28">
         <v>0</v>
       </c>
     </row>
@@ -1008,7 +1006,7 @@
       <c r="D29" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29">
         <v>0.32050000000000001</v>
       </c>
     </row>
@@ -1025,7 +1023,7 @@
       <c r="D30" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30">
         <v>0</v>
       </c>
     </row>
@@ -1042,7 +1040,7 @@
       <c r="D31" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31">
         <v>0</v>
       </c>
     </row>
@@ -1059,7 +1057,7 @@
       <c r="D32" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32" s="3">
         <v>0.39700000000000002</v>
       </c>
     </row>
@@ -1076,7 +1074,7 @@
       <c r="D33" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33">
         <v>0</v>
       </c>
     </row>
@@ -1093,7 +1091,7 @@
       <c r="D34" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E34">
         <v>0</v>
       </c>
     </row>
@@ -2640,7 +2638,7 @@
       <c r="D125" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E125" s="5">
+      <c r="E125" s="3">
         <v>0.78300000000000003</v>
       </c>
     </row>
@@ -2844,7 +2842,7 @@
       <c r="D137" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E137" s="5">
+      <c r="E137" s="3">
         <v>0.83599999999999997</v>
       </c>
     </row>
@@ -3303,7 +3301,7 @@
       <c r="D164" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E164" s="5">
+      <c r="E164" s="3">
         <v>0.497</v>
       </c>
     </row>
@@ -3575,7 +3573,7 @@
       <c r="D180" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E180" s="5">
+      <c r="E180" s="3">
         <v>3.3000000000000002E-2</v>
       </c>
     </row>

</xml_diff>